<commit_message>
description card and contribution workflow
</commit_message>
<xml_diff>
--- a/backend/MPD_Database_Final.xlsx
+++ b/backend/MPD_Database_Final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\syeda\OneDrive\Desktop\ETS\ProductDevelopmentMaps\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A68901-AED1-46ED-9016-652D1F3C143A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221222DC-4F48-42C1-B1BF-55DB488A435B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4170" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4170" uniqueCount="519">
   <si>
     <t>name</t>
   </si>
@@ -1580,6 +1580,9 @@
   </si>
   <si>
     <t>#00747d</t>
+  </si>
+  <si>
+    <t>#c65812</t>
   </si>
 </sst>
 </file>
@@ -13774,7 +13777,7 @@
         <v>366</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
@@ -13917,7 +13920,7 @@
         <v>366</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>432</v>

</xml_diff>